<commit_message>
Site-wide period picker: home dashboard for every month, carried to reports and cards
- Home dashboard Period picker, Nov 2024 to Oct 2026 to date, built per month from the ledger (dashboard_months.py); September validated against the model
- Picked month carries through the visit (sessionStorage / ?period=): report pages, cards and featured charts; reports without that month fall back and say so
- Balance sheet, cash flow and export pack for September 2026 only; other months say so
- History headcount and October hours fixed so utilisation stays believable
- Report pages load reports-data.js once

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/media/exports/reports/2025-10/calls.xlsx
+++ b/media/exports/reports/2025-10/calls.xlsx
@@ -690,7 +690,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Period: October 2025 · Data status: Sep 2025 locked · Oct 2025 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 6:29pm</t>
+          <t>Period: October 2025 · Data status: Sep 2025 locked · Oct 2025 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 11:41pm</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>September 781</t>
+          <t>September 756</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>428 calls to voicemail</t>
+          <t>407 calls to voicemail</t>
         </is>
       </c>
     </row>
@@ -780,7 +780,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>298 answered calls</t>
+          <t>304 answered calls</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
     <row r="33" ht="45" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>792 calls for help came in during October. While the line was staffed, 81.9% were answered (target 90.0%); 54.0% of all calls came outside staffed hours and went to voicemail. The busiest time was 5 to 8pm (151 calls).</t>
+          <t>770 calls for help came in during October. While the line was staffed, 83.7% were answered (target 90.0%); 52.9% of all calls came outside staffed hours and went to voicemail. The busiest time was 5 to 8pm (134 calls).</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>151 calls came between 5 and 8pm, when no-one is on the line. 66 callers hung up waiting while the line was staffed.</t>
+          <t>134 calls came between 5 and 8pm, when no-one is on the line. 59 callers hung up waiting while the line was staffed.</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 calls.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 6:29pm&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 calls.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 11:41pm&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1013,7 +1013,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Period: October 2025 · Data status: Sep 2025 locked · Oct 2025 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 6:29pm</t>
+          <t>Period: October 2025 · Data status: Sep 2025 locked · Oct 2025 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 11:41pm</t>
         </is>
       </c>
     </row>
@@ -1052,10 +1052,10 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>792</v>
+        <v>770</v>
       </c>
       <c r="C8" s="13" t="n">
-        <v>781</v>
+        <v>756</v>
       </c>
     </row>
     <row r="9">
@@ -1065,10 +1065,10 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C9" s="13" t="n">
-        <v>373</v>
+        <v>359</v>
       </c>
     </row>
     <row r="10">
@@ -1078,10 +1078,10 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="C10" s="13" t="n">
-        <v>316</v>
+        <v>307</v>
       </c>
     </row>
     <row r="11">
@@ -1150,10 +1150,10 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>792</v>
+        <v>770</v>
       </c>
       <c r="C18" s="13" t="n">
-        <v>781</v>
+        <v>756</v>
       </c>
     </row>
     <row r="19">
@@ -1163,10 +1163,10 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C19" s="13" t="n">
-        <v>373</v>
+        <v>359</v>
       </c>
     </row>
     <row r="20">
@@ -1176,10 +1176,10 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="C20" s="13" t="n">
-        <v>316</v>
+        <v>307</v>
       </c>
     </row>
     <row r="21">
@@ -1248,10 +1248,10 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>792</v>
+        <v>770</v>
       </c>
       <c r="C28" s="13" t="n">
-        <v>781</v>
+        <v>756</v>
       </c>
     </row>
     <row r="29">
@@ -1261,10 +1261,10 @@
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C29" s="13" t="n">
-        <v>373</v>
+        <v>359</v>
       </c>
     </row>
     <row r="30">
@@ -1274,10 +1274,10 @@
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="C30" s="13" t="n">
-        <v>316</v>
+        <v>307</v>
       </c>
     </row>
     <row r="31">
@@ -1346,10 +1346,10 @@
         </is>
       </c>
       <c r="B38" s="13" t="n">
-        <v>792</v>
+        <v>770</v>
       </c>
       <c r="C38" s="13" t="n">
-        <v>781</v>
+        <v>756</v>
       </c>
     </row>
     <row r="39">
@@ -1359,10 +1359,10 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C39" s="13" t="n">
-        <v>373</v>
+        <v>359</v>
       </c>
     </row>
     <row r="40">
@@ -1372,10 +1372,10 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="C40" s="13" t="n">
-        <v>316</v>
+        <v>307</v>
       </c>
     </row>
     <row r="41">
@@ -1439,7 +1439,7 @@
         </is>
       </c>
       <c r="B48" s="13" t="n">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="49">
@@ -1501,7 +1501,7 @@
         </is>
       </c>
       <c r="B57" s="13" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="58">
@@ -1511,7 +1511,7 @@
         </is>
       </c>
       <c r="B58" s="13" t="n">
-        <v>61</v>
+        <v>69</v>
       </c>
     </row>
     <row r="59">
@@ -1563,7 +1563,7 @@
         </is>
       </c>
       <c r="B66" s="13" t="n">
-        <v>119</v>
+        <v>108</v>
       </c>
     </row>
     <row r="67">
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="B67" s="13" t="n">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="68">
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="B75" s="13" t="n">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="76">
@@ -1635,7 +1635,7 @@
         </is>
       </c>
       <c r="B76" s="13" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="77">
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="B84" s="13" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="85">
@@ -1697,7 +1697,7 @@
         </is>
       </c>
       <c r="B85" s="13" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="86">
@@ -1749,7 +1749,7 @@
         </is>
       </c>
       <c r="B93" s="13" t="n">
-        <v>151</v>
+        <v>134</v>
       </c>
     </row>
     <row r="94">
@@ -1811,7 +1811,7 @@
         </is>
       </c>
       <c r="B102" s="13" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
     </row>
     <row r="103">
@@ -1851,7 +1851,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 calls.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 6:29pm&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 calls.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 11:41pm&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1899,7 +1899,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Period: October 2025 · Data status: Sep 2025 locked · Oct 2025 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 6:29pm</t>
+          <t>Period: October 2025 · Data status: Sep 2025 locked · Oct 2025 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 11:41pm</t>
         </is>
       </c>
     </row>
@@ -1948,13 +1948,13 @@
         </is>
       </c>
       <c r="C6" s="13" t="n">
-        <v>659</v>
+        <v>685</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>312</v>
+        <v>329</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>281</v>
+        <v>299</v>
       </c>
       <c r="F6" s="14">
         <f>IF(D6=0,"",E6/D6)</f>
@@ -1973,13 +1973,13 @@
         </is>
       </c>
       <c r="C7" s="13" t="n">
-        <v>655</v>
+        <v>633</v>
       </c>
       <c r="D7" s="13" t="n">
-        <v>320</v>
+        <v>307</v>
       </c>
       <c r="E7" s="13" t="n">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="F7" s="14">
         <f>IF(D7=0,"",E7/D7)</f>
@@ -1998,10 +1998,10 @@
         </is>
       </c>
       <c r="C8" s="13" t="n">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="E8" s="13" t="n">
         <v>284</v>
@@ -2023,13 +2023,13 @@
         </is>
       </c>
       <c r="C9" s="13" t="n">
-        <v>714</v>
+        <v>690</v>
       </c>
       <c r="D9" s="13" t="n">
         <v>324</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F9" s="14">
         <f>IF(D9=0,"",E9/D9)</f>
@@ -2048,13 +2048,13 @@
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>683</v>
+        <v>664</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="E10" s="13" t="n">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="F10" s="14">
         <f>IF(D10=0,"",E10/D10)</f>
@@ -2073,13 +2073,13 @@
         </is>
       </c>
       <c r="C11" s="13" t="n">
-        <v>725</v>
+        <v>685</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>340</v>
+        <v>311</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>295</v>
+        <v>284</v>
       </c>
       <c r="F11" s="14">
         <f>IF(D11=0,"",E11/D11)</f>
@@ -2098,13 +2098,13 @@
         </is>
       </c>
       <c r="C12" s="13" t="n">
-        <v>620</v>
+        <v>629</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>297</v>
+        <v>286</v>
       </c>
       <c r="E12" s="13" t="n">
-        <v>262</v>
+        <v>246</v>
       </c>
       <c r="F12" s="14">
         <f>IF(D12=0,"",E12/D12)</f>
@@ -2123,13 +2123,13 @@
         </is>
       </c>
       <c r="C13" s="13" t="n">
-        <v>754</v>
+        <v>724</v>
       </c>
       <c r="D13" s="13" t="n">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="E13" s="13" t="n">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="F13" s="14">
         <f>IF(D13=0,"",E13/D13)</f>
@@ -2148,13 +2148,13 @@
         </is>
       </c>
       <c r="C14" s="13" t="n">
-        <v>783</v>
+        <v>820</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>398</v>
+        <v>389</v>
       </c>
       <c r="E14" s="13" t="n">
-        <v>339</v>
+        <v>330</v>
       </c>
       <c r="F14" s="14">
         <f>IF(D14=0,"",E14/D14)</f>
@@ -2173,13 +2173,13 @@
         </is>
       </c>
       <c r="C15" s="13" t="n">
-        <v>871</v>
+        <v>909</v>
       </c>
       <c r="D15" s="13" t="n">
-        <v>428</v>
+        <v>477</v>
       </c>
       <c r="E15" s="13" t="n">
-        <v>362</v>
+        <v>402</v>
       </c>
       <c r="F15" s="14">
         <f>IF(D15=0,"",E15/D15)</f>
@@ -2198,13 +2198,13 @@
         </is>
       </c>
       <c r="C16" s="13" t="n">
-        <v>852</v>
+        <v>826</v>
       </c>
       <c r="D16" s="13" t="n">
-        <v>431</v>
+        <v>388</v>
       </c>
       <c r="E16" s="13" t="n">
-        <v>369</v>
+        <v>327</v>
       </c>
       <c r="F16" s="14">
         <f>IF(D16=0,"",E16/D16)</f>
@@ -2223,13 +2223,13 @@
         </is>
       </c>
       <c r="C17" s="13" t="n">
-        <v>781</v>
+        <v>756</v>
       </c>
       <c r="D17" s="13" t="n">
-        <v>373</v>
+        <v>359</v>
       </c>
       <c r="E17" s="13" t="n">
-        <v>316</v>
+        <v>307</v>
       </c>
       <c r="F17" s="14">
         <f>IF(D17=0,"",E17/D17)</f>
@@ -2248,13 +2248,13 @@
         </is>
       </c>
       <c r="C18" s="13" t="n">
-        <v>792</v>
+        <v>770</v>
       </c>
       <c r="D18" s="13" t="n">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E18" s="13" t="n">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="F18" s="14">
         <f>IF(D18=0,"",E18/D18)</f>
@@ -2267,7 +2267,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 calls.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 6:29pm&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 calls.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 11:41pm&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>